<commit_message>
cleaning up index and adding index column
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54BDE654-CDA6-7E48-B67E-70C29C6C84E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FF98C2-538C-B043-877E-D6537898227E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="18500" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12380" yWindow="-19580" windowWidth="18500" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>week</t>
   </si>
@@ -105,6 +105,21 @@
   </si>
   <si>
     <t>practice-activities/main-version/pa7-wrangling.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa4-friend.qmd</t>
+  </si>
+  <si>
+    <t>labs/main-version/lab1-hello-code.qmd</t>
+  </si>
+  <si>
+    <t>labs/main-version/lab2-r-is-friend.qmd</t>
+  </si>
+  <si>
+    <t>preparation</t>
+  </si>
+  <si>
+    <t>reading/week-5.qmd</t>
   </si>
 </sst>
 </file>
@@ -410,18 +425,18 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="3" max="3" width="31.6640625" customWidth="1"/>
-    <col min="4" max="4" width="32.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.33203125" customWidth="1"/>
-    <col min="7" max="7" width="27.5" customWidth="1"/>
-    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="3" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="32.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" customWidth="1"/>
+    <col min="7" max="7" width="31.33203125" customWidth="1"/>
+    <col min="8" max="8" width="27.5" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,20 +447,23 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -455,8 +473,9 @@
       <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -464,8 +483,12 @@
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D3" s="1"/>
+      <c r="H3" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -475,8 +498,9 @@
       <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -484,9 +508,12 @@
         <v>2</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D5" s="1"/>
+      <c r="H5" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -496,12 +523,13 @@
       <c r="C6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="1"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -509,12 +537,13 @@
         <v>2</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="1"/>
       <c r="E7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="F7" s="3"/>
       <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1">
         <v>4</v>
       </c>
@@ -524,12 +553,13 @@
       <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="1"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1">
         <v>4</v>
       </c>
@@ -539,12 +569,16 @@
       <c r="C9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="1"/>
       <c r="E9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1">
         <v>5</v>
       </c>
@@ -554,12 +588,15 @@
       <c r="C10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
         <v>5</v>
       </c>
@@ -567,13 +604,14 @@
         <v>2</v>
       </c>
       <c r="C11" s="1"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="1"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
         <v>6</v>
       </c>
@@ -583,13 +621,14 @@
       <c r="C12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="F12" s="3" t="s">
+      <c r="D12" s="1"/>
+      <c r="E12" s="3"/>
+      <c r="G12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1">
         <v>6</v>
       </c>
@@ -597,8 +636,9 @@
         <v>2</v>
       </c>
       <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">
         <v>7</v>
       </c>
@@ -608,8 +648,9 @@
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">
         <v>7</v>
       </c>
@@ -617,8 +658,9 @@
         <v>2</v>
       </c>
       <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">
         <v>8</v>
       </c>
@@ -628,8 +670,9 @@
       <c r="C16" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -637,8 +680,9 @@
         <v>2</v>
       </c>
       <c r="C17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
         <v>9</v>
       </c>
@@ -648,8 +692,9 @@
       <c r="C18" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
         <v>9</v>
       </c>
@@ -657,8 +702,9 @@
         <v>2</v>
       </c>
       <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
         <v>10</v>
       </c>
@@ -668,8 +714,9 @@
       <c r="C20" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D20" s="1"/>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1">
         <v>10</v>
       </c>
@@ -679,8 +726,9 @@
       <c r="C21" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1">
         <v>11</v>
       </c>
@@ -690,20 +738,21 @@
       <c r="C22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="4"/>
       <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
         <v>11</v>
       </c>
       <c r="B23" s="1">
         <v>2</v>
       </c>
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="1">
         <v>12</v>
       </c>
@@ -713,18 +762,19 @@
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="4"/>
-    </row>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D24" s="1"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1">
         <v>12</v>
       </c>
       <c r="B25" s="1">
         <v>2</v>
       </c>
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1">
         <v>13</v>
       </c>
@@ -734,18 +784,19 @@
       <c r="C26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="4"/>
-    </row>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D26" s="1"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
         <v>13</v>
       </c>
       <c r="B27" s="1">
         <v>2</v>
       </c>
-      <c r="G27" s="1"/>
-    </row>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
         <v>14</v>
       </c>
@@ -755,66 +806,67 @@
       <c r="C28" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="2"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="4"/>
       <c r="F28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1">
         <v>14</v>
       </c>
       <c r="B29" s="1">
         <v>2</v>
       </c>
-      <c r="D29" s="5"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1">
         <v>15</v>
       </c>
       <c r="B30" s="1">
         <v>1</v>
       </c>
-      <c r="D30" s="6"/>
-      <c r="G30" s="1"/>
-    </row>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E30" s="6"/>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1">
         <v>15</v>
       </c>
       <c r="B31" s="1">
         <v>2</v>
       </c>
-      <c r="D31" s="5"/>
-      <c r="G31" s="1"/>
-    </row>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G32" s="1"/>
-    </row>
-    <row r="33" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D33" s="5"/>
-    </row>
-    <row r="34" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D35" s="5"/>
-      <c r="G35" s="1"/>
-    </row>
-    <row r="36" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D36" s="5"/>
-      <c r="G36" s="1"/>
-    </row>
-    <row r="37" spans="4:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D37" s="1"/>
-    </row>
-    <row r="39" spans="4:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="D39" s="2"/>
+      <c r="E31" s="5"/>
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E35" s="5"/>
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E36" s="5"/>
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E37" s="1"/>
+    </row>
+    <row r="39" spans="5:8" ht="13" x14ac:dyDescent="0.15">
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="4:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="D40" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="5:8" ht="13" x14ac:dyDescent="0.15">
+      <c r="E40" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
add links to unit 1 readings and assignments
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FF98C2-538C-B043-877E-D6537898227E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B84F73-318C-B746-94A1-DE52D9949AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12380" yWindow="-19580" windowWidth="18500" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>week</t>
   </si>
@@ -120,6 +120,39 @@
   </si>
   <si>
     <t>reading/week-5.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa1-tracing.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa2-indexing.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa3-control-flow.qmd</t>
+  </si>
+  <si>
+    <t>labs/main-version/lab3-control-flow.qmd</t>
+  </si>
+  <si>
+    <t>practice exam</t>
+  </si>
+  <si>
+    <t>Computer is Friend</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>https://r-is-your-friend.github.io/course-pack/00-setup.html</t>
+  </si>
+  <si>
+    <t>https://r-is-your-friend.github.io/course-pack/01-what-is-code.html</t>
+  </si>
+  <si>
+    <t>https://r-is-your-friend.github.io/course-pack/02-r-is-friend.html</t>
+  </si>
+  <si>
+    <t>https://r-is-your-friend.github.io/course-pack/03-control-flow.html</t>
   </si>
 </sst>
 </file>
@@ -425,18 +458,18 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="3" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="32.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.33203125" customWidth="1"/>
-    <col min="7" max="7" width="31.33203125" customWidth="1"/>
-    <col min="8" max="8" width="27.5" customWidth="1"/>
-    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="3" max="5" width="31.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.33203125" customWidth="1"/>
+    <col min="8" max="8" width="41.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.5" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,426 +480,559 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="H1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="H3" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="I4" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="s">
+    <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1">
-        <v>2</v>
-      </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="H5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="I6" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
+    <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="1">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1">
-        <v>2</v>
-      </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="3"/>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="F7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="1">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1">
         <v>4</v>
       </c>
       <c r="B9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="1">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="1">
-        <v>5</v>
-      </c>
-      <c r="B10" s="1">
-        <v>1</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="3"/>
+      <c r="D10" s="1">
+        <v>2</v>
+      </c>
+      <c r="E10" s="1"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
+      <c r="H10" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
         <v>5</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B12" s="1">
-        <v>1</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="3"/>
-      <c r="G12" s="3" t="s">
-        <v>23</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1">
         <v>6</v>
       </c>
       <c r="B13" s="1">
-        <v>2</v>
-      </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="F13" s="3"/>
+      <c r="H13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="1">
-        <v>1</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">
         <v>7</v>
       </c>
       <c r="B15" s="1">
-        <v>2</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B16" s="1">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
         <v>8</v>
       </c>
       <c r="B17" s="1">
-        <v>2</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="1">
-        <v>1</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
         <v>9</v>
       </c>
       <c r="B19" s="1">
-        <v>2</v>
-      </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1">
+        <v>2</v>
+      </c>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20" s="1">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1">
+        <v>2</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1">
         <v>10</v>
       </c>
       <c r="B21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2</v>
+      </c>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="1">
+        <v>10</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="1">
-        <v>11</v>
-      </c>
-      <c r="B22" s="1">
-        <v>1</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D22" s="1">
+        <v>2</v>
+      </c>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
         <v>11</v>
       </c>
       <c r="B23" s="1">
-        <v>2</v>
-      </c>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="1">
+        <v>3</v>
+      </c>
+      <c r="E23" s="1"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" s="1">
-        <v>1</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="D24" s="1">
+        <v>3</v>
+      </c>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1">
         <v>12</v>
       </c>
       <c r="B25" s="1">
-        <v>2</v>
-      </c>
-      <c r="E25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" s="1">
+        <v>3</v>
+      </c>
+      <c r="E25" s="1"/>
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" s="1">
-        <v>1</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="1"/>
-      <c r="E26" s="4"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1">
+        <v>3</v>
+      </c>
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
         <v>13</v>
       </c>
       <c r="B27" s="1">
-        <v>2</v>
-      </c>
-      <c r="H27" s="1"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="1">
+        <v>3</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B28" s="1">
-        <v>1</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3</v>
+      </c>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1">
         <v>14</v>
       </c>
       <c r="B29" s="1">
-        <v>2</v>
-      </c>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D29" s="1">
+        <v>3</v>
+      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B30" s="1">
-        <v>1</v>
-      </c>
-      <c r="E30" s="6"/>
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1">
+        <v>3</v>
+      </c>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1">
         <v>15</v>
       </c>
       <c r="B31" s="1">
-        <v>2</v>
-      </c>
-      <c r="E31" s="5"/>
-      <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E35" s="5"/>
-      <c r="H35" s="1"/>
-    </row>
-    <row r="36" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E36" s="5"/>
-      <c r="H36" s="1"/>
-    </row>
-    <row r="37" spans="5:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="E37" s="1"/>
-    </row>
-    <row r="39" spans="5:8" ht="13" x14ac:dyDescent="0.15">
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-    </row>
-    <row r="40" spans="5:8" ht="13" x14ac:dyDescent="0.15">
-      <c r="E40" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D31" s="1">
+        <v>3</v>
+      </c>
+      <c r="F31" s="6"/>
+      <c r="I31" s="1"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="1">
+        <v>15</v>
+      </c>
+      <c r="B32" s="1">
+        <v>2</v>
+      </c>
+      <c r="D32" s="1">
+        <v>3</v>
+      </c>
+      <c r="F32" s="5"/>
+      <c r="I32" s="1"/>
+    </row>
+    <row r="33" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I33" s="1"/>
+    </row>
+    <row r="34" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F34" s="5"/>
+    </row>
+    <row r="35" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F36" s="5"/>
+      <c r="I36" s="1"/>
+    </row>
+    <row r="37" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F37" s="5"/>
+      <c r="I37" s="1"/>
+    </row>
+    <row r="38" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F38" s="1"/>
+    </row>
+    <row r="40" spans="6:9" ht="13" x14ac:dyDescent="0.15">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="6:9" ht="13" x14ac:dyDescent="0.15">
+      <c r="F41" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
add slides and handout to excel file, render site
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B84F73-318C-B746-94A1-DE52D9949AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6EED49-4B81-A642-9467-73A8830BB57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>week</t>
   </si>
@@ -153,6 +153,12 @@
   </si>
   <si>
     <t>https://r-is-your-friend.github.io/course-pack/03-control-flow.html</t>
+  </si>
+  <si>
+    <t>slides/01-tracing.qmd</t>
+  </si>
+  <si>
+    <t>handouts/01-tracing.qmd</t>
   </si>
 </sst>
 </file>
@@ -461,7 +467,8 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="3" max="5" width="31.6640625" customWidth="1"/>
+    <col min="3" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="51.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.33203125" customWidth="1"/>
     <col min="8" max="8" width="41.6640625" bestFit="1" customWidth="1"/>
@@ -539,6 +546,12 @@
       <c r="E3" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="F3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="H3" s="3" t="s">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
adjust lag for week label
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6EED49-4B81-A642-9467-73A8830BB57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9FD1A87-559B-A442-8EC8-9C2CCCDCDAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>week</t>
   </si>
@@ -59,9 +59,6 @@
     <t>day</t>
   </si>
   <si>
-    <t>What is Code?</t>
-  </si>
-  <si>
     <t>R is friend</t>
   </si>
   <si>
@@ -137,28 +134,25 @@
     <t>practice exam</t>
   </si>
   <si>
-    <t>Computer is Friend</t>
-  </si>
-  <si>
     <t>unit</t>
   </si>
   <si>
-    <t>https://r-is-your-friend.github.io/course-pack/00-setup.html</t>
-  </si>
-  <si>
-    <t>https://r-is-your-friend.github.io/course-pack/01-what-is-code.html</t>
-  </si>
-  <si>
-    <t>https://r-is-your-friend.github.io/course-pack/02-r-is-friend.html</t>
-  </si>
-  <si>
-    <t>https://r-is-your-friend.github.io/course-pack/03-control-flow.html</t>
-  </si>
-  <si>
     <t>slides/01-tracing.qmd</t>
   </si>
   <si>
     <t>handouts/01-tracing.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-1.qmd</t>
+  </si>
+  <si>
+    <t>Computer is Friend &amp; What is Code?</t>
+  </si>
+  <si>
+    <t>reading/week-2.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-3.qmd</t>
   </si>
 </sst>
 </file>
@@ -464,7 +458,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="3" max="4" width="31.6640625" customWidth="1"/>
@@ -487,10 +481,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -505,71 +499,69 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="F2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
       <c r="D3" s="1">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>29</v>
+      <c r="E3" s="1"/>
+      <c r="I3" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="I4" s="3" t="s">
-        <v>25</v>
+      <c r="E4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -577,77 +569,76 @@
         <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C5" s="1"/>
       <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>30</v>
+      <c r="E5" s="1"/>
+      <c r="I5" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="I6" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="E6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1">
         <v>3</v>
       </c>
       <c r="B7" s="1">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C7" s="1"/>
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>31</v>
       </c>
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="D8" s="1">
         <v>1</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="I8" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="H8" s="3"/>
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -655,26 +646,29 @@
         <v>4</v>
       </c>
       <c r="B9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
@@ -682,13 +676,12 @@
       <c r="D10" s="1">
         <v>2</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I10" s="3"/>
+      <c r="H10" s="3"/>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -696,38 +689,37 @@
         <v>5</v>
       </c>
       <c r="B11" s="1">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C11" s="1"/>
       <c r="D11" s="1">
         <v>2</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B12" s="1">
-        <v>2</v>
-      </c>
-      <c r="C12" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="D12" s="1">
         <v>2</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="H12" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -735,29 +727,24 @@
         <v>6</v>
       </c>
       <c r="B13" s="1">
-        <v>1</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C13" s="1"/>
       <c r="D13" s="1">
         <v>2</v>
       </c>
       <c r="E13" s="1"/>
-      <c r="F13" s="3"/>
-      <c r="H13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J13" s="3"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="1">
-        <v>2</v>
-      </c>
-      <c r="C14" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="D14" s="1">
         <v>2</v>
       </c>
@@ -768,11 +755,9 @@
         <v>7</v>
       </c>
       <c r="B15" s="1">
-        <v>1</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C15" s="1"/>
       <c r="D15" s="1">
         <v>2</v>
       </c>
@@ -780,12 +765,14 @@
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B16" s="1">
-        <v>2</v>
-      </c>
-      <c r="C16" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="D16" s="1">
         <v>2</v>
       </c>
@@ -796,11 +783,9 @@
         <v>8</v>
       </c>
       <c r="B17" s="1">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C17" s="1"/>
       <c r="D17" s="1">
         <v>2</v>
       </c>
@@ -808,12 +793,14 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B18" s="1">
-        <v>2</v>
-      </c>
-      <c r="C18" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="D18" s="1">
         <v>2</v>
       </c>
@@ -824,11 +811,9 @@
         <v>9</v>
       </c>
       <c r="B19" s="1">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>17</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C19" s="1"/>
       <c r="D19" s="1">
         <v>2</v>
       </c>
@@ -836,12 +821,14 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B20" s="1">
-        <v>2</v>
-      </c>
-      <c r="C20" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="D20" s="1">
         <v>2</v>
       </c>
@@ -852,7 +839,7 @@
         <v>10</v>
       </c>
       <c r="B21" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>18</v>
@@ -864,47 +851,48 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" s="1"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
         <v>11</v>
       </c>
       <c r="B23" s="1">
-        <v>1</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D23" s="1">
         <v>3</v>
       </c>
-      <c r="E23" s="1"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B24" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="D24" s="1">
         <v>3</v>
       </c>
+      <c r="E24" s="1"/>
       <c r="F24" s="4"/>
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -912,27 +900,27 @@
         <v>12</v>
       </c>
       <c r="B25" s="1">
-        <v>1</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D25" s="1">
         <v>3</v>
       </c>
-      <c r="E25" s="1"/>
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B26" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D26" s="1">
         <v>3</v>
       </c>
+      <c r="E26" s="1"/>
       <c r="F26" s="4"/>
     </row>
     <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -940,112 +928,96 @@
         <v>13</v>
       </c>
       <c r="B27" s="1">
-        <v>1</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D27" s="1">
         <v>3</v>
       </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="4"/>
+      <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D28" s="1">
         <v>3</v>
       </c>
-      <c r="I28" s="1"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1">
         <v>14</v>
       </c>
       <c r="B29" s="1">
-        <v>1</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D29" s="1">
         <v>3</v>
       </c>
-      <c r="E29" s="3"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
+      <c r="F29" s="5"/>
     </row>
     <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B30" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="1">
         <v>3</v>
       </c>
-      <c r="F30" s="5"/>
+      <c r="F30" s="6"/>
+      <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1">
         <v>15</v>
       </c>
       <c r="B31" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="1">
         <v>3</v>
       </c>
-      <c r="F31" s="6"/>
+      <c r="F31" s="5"/>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="1">
-        <v>15</v>
-      </c>
-      <c r="B32" s="1">
-        <v>2</v>
-      </c>
-      <c r="D32" s="1">
-        <v>3</v>
-      </c>
-      <c r="F32" s="5"/>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="I33" s="1"/>
+      <c r="F33" s="5"/>
     </row>
     <row r="34" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F34" s="5"/>
+      <c r="F34" s="2"/>
     </row>
     <row r="35" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F35" s="2"/>
+      <c r="F35" s="5"/>
+      <c r="I35" s="1"/>
     </row>
     <row r="36" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="F36" s="5"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F37" s="5"/>
-      <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="6:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F38" s="1"/>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="39" spans="6:9" ht="13" x14ac:dyDescent="0.15">
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
     </row>
     <row r="40" spans="6:9" ht="13" x14ac:dyDescent="0.15">
       <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-    </row>
-    <row r="41" spans="6:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="F41" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
add functions to week 3 content
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9FD1A87-559B-A442-8EC8-9C2CCCDCDAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46F001C-308D-6641-9BE7-315949BF9D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>week</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Unit 2 Assessment</t>
   </si>
   <si>
-    <t>Functions</t>
-  </si>
-  <si>
     <t>Functions and Regression</t>
   </si>
   <si>
@@ -128,9 +125,6 @@
     <t>practice-activities/main-version/pa3-control-flow.qmd</t>
   </si>
   <si>
-    <t>labs/main-version/lab3-control-flow.qmd</t>
-  </si>
-  <si>
     <t>practice exam</t>
   </si>
   <si>
@@ -152,7 +146,19 @@
     <t>reading/week-2.qmd</t>
   </si>
   <si>
-    <t>reading/week-3.qmd</t>
+    <t>Writing Simple Functions</t>
+  </si>
+  <si>
+    <t>Writing More Complex Functions</t>
+  </si>
+  <si>
+    <t>reading/week-3a.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-3b.qmd</t>
+  </si>
+  <si>
+    <t>labs/main-version/lab3-functions-control-flow.qmd</t>
   </si>
 </sst>
 </file>
@@ -481,10 +487,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -499,7 +505,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -510,22 +516,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -541,7 +547,7 @@
       </c>
       <c r="E3" s="1"/>
       <c r="I3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -558,10 +564,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -577,7 +583,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="I5" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -599,7 +605,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -610,15 +616,19 @@
       <c r="B7" s="1">
         <v>2</v>
       </c>
-      <c r="C7" s="1"/>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -658,7 +668,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -677,7 +687,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -718,7 +728,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -857,7 +867,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>
@@ -887,7 +897,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D24" s="1">
         <v>3</v>
@@ -943,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D28" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
adding pas and data + link to data index
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10FC419-E248-0743-B56C-F6A3C3DD60CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B1A40A6-DD19-B040-82E4-29F086516396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>week</t>
   </si>
@@ -98,9 +98,6 @@
     <t>Unit 3 Assessment</t>
   </si>
   <si>
-    <t>practice-activities/main-version/pa7-wrangling.qmd</t>
-  </si>
-  <si>
     <t>practice-activities/main-version/pa4-friend.qmd</t>
   </si>
   <si>
@@ -174,6 +171,12 @@
   </si>
   <si>
     <t>reading/week-9.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa6-wrangling.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/main-version/pa7-pivot.qmd</t>
   </si>
 </sst>
 </file>
@@ -502,10 +505,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -520,7 +523,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -531,22 +534,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -562,7 +565,7 @@
       </c>
       <c r="E3" s="1"/>
       <c r="I3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -579,10 +582,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -598,7 +601,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="I5" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -615,12 +618,12 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -632,18 +635,18 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -680,12 +683,12 @@
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -704,7 +707,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -743,11 +746,11 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -778,7 +781,10 @@
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -808,7 +814,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -838,7 +844,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -892,7 +898,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
move a couple things around and clean render with versioning
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDE3B22-2166-A840-9C99-9FBAC137ED66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6865C709-6AEA-DA4A-881F-229F849B9691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>week</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>practice-activities/instructions/pa7-pivot.qmd</t>
+  </si>
+  <si>
+    <t>labs/instructions/lab9-murder.qmd</t>
   </si>
 </sst>
 </file>
@@ -859,6 +862,9 @@
         <v>2</v>
       </c>
       <c r="E19" s="1"/>
+      <c r="I19" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">

</xml_diff>

<commit_message>
split week 8 reading (rendered a bunch of other stuff in the process)
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6865C709-6AEA-DA4A-881F-229F849B9691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BE1EB8-9496-A147-A733-C598298B141A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>week</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Data Wrangling Continued</t>
   </si>
   <si>
-    <t>Joins and Factors</t>
-  </si>
-  <si>
     <t>Strings and Dates</t>
   </si>
   <si>
@@ -167,9 +164,6 @@
     <t>reading/week-7.qmd</t>
   </si>
   <si>
-    <t>reading/week-8.qmd</t>
-  </si>
-  <si>
     <t>reading/week-9.qmd</t>
   </si>
   <si>
@@ -180,6 +174,18 @@
   </si>
   <si>
     <t>labs/instructions/lab9-murder.qmd</t>
+  </si>
+  <si>
+    <t>Joins</t>
+  </si>
+  <si>
+    <t>Factors</t>
+  </si>
+  <si>
+    <t>reading/week-8a.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-8b.qmd</t>
   </si>
 </sst>
 </file>
@@ -508,10 +514,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -526,7 +532,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -537,22 +543,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -568,7 +574,7 @@
       </c>
       <c r="E3" s="1"/>
       <c r="I3" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -585,10 +591,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -604,7 +610,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="I5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -621,12 +627,12 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -638,18 +644,18 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -686,12 +692,12 @@
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -710,7 +716,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -749,11 +755,11 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -784,10 +790,10 @@
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -811,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D16" s="1">
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -827,11 +833,15 @@
       <c r="B17" s="1">
         <v>2</v>
       </c>
-      <c r="C17" s="1"/>
+      <c r="C17" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="D17" s="1">
         <v>2</v>
       </c>
-      <c r="E17" s="1"/>
+      <c r="E17" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
@@ -841,13 +851,13 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" s="1">
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -863,7 +873,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="I19" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -874,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D20" s="1">
         <v>2</v>
@@ -889,7 +899,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D21" s="1">
         <v>2</v>
@@ -904,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>
@@ -934,7 +944,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D24" s="1">
         <v>3</v>
@@ -990,7 +1000,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D28" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
add week 7 in class stuff to index
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BE1EB8-9496-A147-A733-C598298B141A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9C53-A65C-9749-BB49-AA6DBBCC0BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>week</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t>reading/week-8b.qmd</t>
+  </si>
+  <si>
+    <t>handouts/07-handout.qmd</t>
+  </si>
+  <si>
+    <t>code-along/student/07-code-along.qmd</t>
   </si>
 </sst>
 </file>
@@ -792,6 +798,9 @@
       <c r="E14" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="G14" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="H14" s="3" t="s">
         <v>45</v>
       </c>
@@ -808,6 +817,9 @@
         <v>2</v>
       </c>
       <c r="E15" s="1"/>
+      <c r="G15" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">

</xml_diff>

<commit_message>
rought PA and lab 8
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9C53-A65C-9749-BB49-AA6DBBCC0BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032AFC79-D2D5-8C42-B661-2115C1493FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>week</t>
   </si>
@@ -192,6 +192,15 @@
   </si>
   <si>
     <t>code-along/student/07-code-along.qmd</t>
+  </si>
+  <si>
+    <t>code-along/student/08-code-along.qmd</t>
+  </si>
+  <si>
+    <t>labs/instructions/lab8-childcare.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa8-joins.qmd</t>
   </si>
 </sst>
 </file>
@@ -837,6 +846,9 @@
       <c r="E16" s="1" t="s">
         <v>49</v>
       </c>
+      <c r="H16" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
@@ -853,6 +865,12 @@
       </c>
       <c r="E17" s="1" t="s">
         <v>50</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
adding all drafts to index and versioning to previously created pas
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032AFC79-D2D5-8C42-B661-2115C1493FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B0F504-0165-F843-B079-2134904CC078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>week</t>
   </si>
@@ -95,9 +95,6 @@
     <t>Unit 3 Assessment</t>
   </si>
   <si>
-    <t>practice-activities/main-version/pa4-friend.qmd</t>
-  </si>
-  <si>
     <t>labs/main-version/lab1-hello-code.qmd</t>
   </si>
   <si>
@@ -167,9 +164,6 @@
     <t>reading/week-9.qmd</t>
   </si>
   <si>
-    <t>practice-activities/main-version/pa6-wrangling.qmd</t>
-  </si>
-  <si>
     <t>practice-activities/instructions/pa7-pivot.qmd</t>
   </si>
   <si>
@@ -201,6 +195,15 @@
   </si>
   <si>
     <t>practice-activities/instructions/pa8-joins.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa9-strings-dates.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa6-wrangling.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa4-friend.qmd</t>
   </si>
 </sst>
 </file>
@@ -529,10 +532,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -547,7 +550,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -558,22 +561,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -589,7 +592,7 @@
       </c>
       <c r="E3" s="1"/>
       <c r="I3" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -606,10 +609,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -625,7 +628,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="I5" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -642,12 +645,12 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -659,18 +662,18 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -707,12 +710,12 @@
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -731,7 +734,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -770,11 +773,11 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -805,13 +808,13 @@
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -827,7 +830,7 @@
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -838,16 +841,16 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="1">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="1">
-        <v>2</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="H16" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -858,19 +861,19 @@
         <v>2</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="1">
-        <v>2</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="G17" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -887,7 +890,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -902,8 +908,11 @@
         <v>2</v>
       </c>
       <c r="E19" s="1"/>
+      <c r="G19" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="I19" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -944,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
update links in index
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B0F504-0165-F843-B079-2134904CC078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B6928E-9EC3-3B45-911D-CFC53740FFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -95,27 +95,12 @@
     <t>Unit 3 Assessment</t>
   </si>
   <si>
-    <t>labs/main-version/lab1-hello-code.qmd</t>
-  </si>
-  <si>
-    <t>labs/main-version/lab2-r-is-friend.qmd</t>
-  </si>
-  <si>
     <t>preparation</t>
   </si>
   <si>
     <t>reading/week-5.qmd</t>
   </si>
   <si>
-    <t>practice-activities/main-version/pa1-tracing.qmd</t>
-  </si>
-  <si>
-    <t>practice-activities/main-version/pa2-indexing.qmd</t>
-  </si>
-  <si>
-    <t>practice-activities/main-version/pa3-control-flow.qmd</t>
-  </si>
-  <si>
     <t>practice exam</t>
   </si>
   <si>
@@ -149,9 +134,6 @@
     <t>reading/week-3b.qmd</t>
   </si>
   <si>
-    <t>labs/main-version/lab3-functions-control-flow.qmd</t>
-  </si>
-  <si>
     <t>reading/week-4.qmd</t>
   </si>
   <si>
@@ -204,6 +186,24 @@
   </si>
   <si>
     <t>practice-activities/instructions/pa4-friend.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa2-indexing.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa1-tracing.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa3-control-flow.qmd</t>
+  </si>
+  <si>
+    <t>labs/instructions/lab2-r-is-friend.qmd</t>
+  </si>
+  <si>
+    <t>labs/instructions/lab1-hello-code.qmd</t>
+  </si>
+  <si>
+    <t>labs/instructions/lab3-functions-control-flow.qmd</t>
   </si>
 </sst>
 </file>
@@ -532,10 +532,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -550,7 +550,7 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -561,22 +561,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -592,7 +592,7 @@
       </c>
       <c r="E3" s="1"/>
       <c r="I3" s="3" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -609,10 +609,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -628,7 +628,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="I5" s="3" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -645,12 +645,12 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -662,18 +662,18 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -710,12 +710,12 @@
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -734,7 +734,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -773,11 +773,11 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -808,13 +808,13 @@
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -830,7 +830,7 @@
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -841,16 +841,16 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D16" s="1">
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -861,19 +861,19 @@
         <v>2</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="D17" s="1">
-        <v>2</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -890,10 +890,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -909,10 +909,10 @@
       </c>
       <c r="E19" s="1"/>
       <c r="G19" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -953,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
adding data viz and communication content
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erobin17/Documents/scholarship/r-is-your-friend/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B6928E-9EC3-3B45-911D-CFC53740FFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC164B3-C055-054C-B397-37C6B48C81CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>week</t>
   </si>
@@ -204,6 +204,12 @@
   </si>
   <si>
     <t>labs/instructions/lab3-functions-control-flow.qmd</t>
+  </si>
+  <si>
+    <t>reading/week-10.qmd</t>
+  </si>
+  <si>
+    <t>practice-activities/instructions/pa5-dataviz.qmd</t>
   </si>
 </sst>
 </file>
@@ -738,7 +744,9 @@
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -928,7 +936,9 @@
       <c r="D20" s="1">
         <v>2</v>
       </c>
-      <c r="E20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1">

</xml_diff>

<commit_message>
render pa 5 and handout 5 to index
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erobin17/Documents/scholarship/r-is-your-friend/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE13A385-1B3B-7840-8314-D63B2601B0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F50F7B2-156A-EA43-B03A-521F0A8528E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
   <si>
     <t>week</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>handouts/04-handout.qmd</t>
+  </si>
+  <si>
+    <t>handouts/05-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -748,7 +751,9 @@
         <v>21</v>
       </c>
       <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
+      <c r="G10" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="H10" s="3" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
check links for unit 1 content, add code along and slides to homepage
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erobin17/Documents/scholarship/r-is-your-friend/course-assessments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F50F7B2-156A-EA43-B03A-521F0A8528E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C122B915-8325-AC46-8180-E57A076F84D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38760" yWindow="720" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>week</t>
   </si>
@@ -216,6 +216,21 @@
   </si>
   <si>
     <t>handouts/05-handout.qmd</t>
+  </si>
+  <si>
+    <t>code-along/instructions/01-code-along.qmd</t>
+  </si>
+  <si>
+    <t>code-along/instructions/02-code-along.qmd</t>
+  </si>
+  <si>
+    <t>code-along/instructions/03-code-along.qmd</t>
+  </si>
+  <si>
+    <t>slides/02-indexing.qmd</t>
+  </si>
+  <si>
+    <t>slides/03a-control-flow.qmd</t>
   </si>
 </sst>
 </file>
@@ -603,6 +618,9 @@
         <v>1</v>
       </c>
       <c r="E3" s="1"/>
+      <c r="H3" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="I3" s="3" t="s">
         <v>55</v>
       </c>
@@ -623,6 +641,9 @@
       <c r="E4" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="F4" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="H4" s="3" t="s">
         <v>51</v>
       </c>
@@ -639,6 +660,9 @@
         <v>1</v>
       </c>
       <c r="E5" s="1"/>
+      <c r="H5" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="I5" s="3" t="s">
         <v>54</v>
       </c>
@@ -659,7 +683,9 @@
       <c r="E6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>65</v>
+      </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
         <v>53</v>
@@ -684,6 +710,9 @@
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
+      <c r="H7" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="I7" s="3" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
add handouts to main page
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C122B915-8325-AC46-8180-E57A076F84D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967BCF66-9075-C54C-A44C-3718A63C2B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38760" yWindow="720" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>week</t>
   </si>
@@ -110,9 +110,6 @@
     <t>slides/01-tracing.qmd</t>
   </si>
   <si>
-    <t>handouts/01-tracing.qmd</t>
-  </si>
-  <si>
     <t>reading/week-1.qmd</t>
   </si>
   <si>
@@ -231,6 +228,21 @@
   </si>
   <si>
     <t>slides/03a-control-flow.qmd</t>
+  </si>
+  <si>
+    <t>slides/03b-functions.qmd</t>
+  </si>
+  <si>
+    <t>handouts/03a-handout.qmd</t>
+  </si>
+  <si>
+    <t>handouts/03b-handout.qmd</t>
+  </si>
+  <si>
+    <t>handouts/01-handout.qmd</t>
+  </si>
+  <si>
+    <t>handouts/02-handout.qmd</t>
   </si>
 </sst>
 </file>
@@ -588,22 +600,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -619,10 +631,10 @@
       </c>
       <c r="E3" s="1"/>
       <c r="H3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -639,13 +651,16 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -661,10 +676,10 @@
       </c>
       <c r="E5" s="1"/>
       <c r="H5" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -681,14 +696,16 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" s="3"/>
+        <v>64</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="H6" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -700,21 +717,25 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="H7" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -751,14 +772,14 @@
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -781,10 +802,10 @@
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J10" s="3"/>
     </row>
@@ -820,11 +841,11 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -855,13 +876,13 @@
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -877,7 +898,7 @@
       </c>
       <c r="E15" s="1"/>
       <c r="G15" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -888,16 +909,16 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="1">
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -908,19 +929,19 @@
         <v>2</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="1">
         <v>2</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -937,10 +958,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -956,10 +977,10 @@
       </c>
       <c r="E19" s="1"/>
       <c r="G19" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -976,7 +997,7 @@
         <v>2</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1002,7 +1023,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D22" s="1">
         <v>3</v>

</xml_diff>

<commit_message>
9 code along and 8 handout
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atheobol/Documents/Teaching/STAT 1810/course-assessments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/r-revamp/course-assessments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967BCF66-9075-C54C-A44C-3718A63C2B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD56D7A7-6A61-054C-86C2-889D378D7EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>week</t>
   </si>
@@ -243,6 +243,9 @@
   </si>
   <si>
     <t>handouts/02-handout.qmd</t>
+  </si>
+  <si>
+    <t>code-along/student/09-code-along.qmd</t>
   </si>
 </sst>
 </file>
@@ -977,7 +980,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="G19" s="3" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>37</v>
@@ -1014,6 +1017,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="1"/>
+      <c r="G21" s="3"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1">

</xml_diff>